<commit_message>
Update Task 4 sheet layout, separate deposit date, fix file names
</commit_message>
<xml_diff>
--- a/Task4/Task4.xlsx
+++ b/Task4/Task4.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U6"/>
+  <dimension ref="A1:S6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -434,16 +434,14 @@
     <col width="12" customWidth="1" min="15" max="15"/>
     <col width="12" customWidth="1" min="16" max="16"/>
     <col width="12" customWidth="1" min="17" max="17"/>
-    <col width="13" customWidth="1" min="18" max="18"/>
-    <col width="12" customWidth="1" min="19" max="19"/>
-    <col width="22" customWidth="1" min="20" max="20"/>
-    <col width="18" customWidth="1" min="21" max="21"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="13" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>source_file</t>
+          <t>source file</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
@@ -458,32 +456,32 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>invoice_number</t>
+          <t>invoice number</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>invoice_date</t>
+          <t>invoice date</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>due_date</t>
+          <t>due date</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>event_date</t>
+          <t>event date</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>customer_reference</t>
+          <t>customer reference</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>payment_terms</t>
+          <t>payment terms</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
@@ -498,24 +496,24 @@
       </c>
       <c r="L1" t="inlineStr">
         <is>
+          <t>tax amount</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>delivery</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>tax rate</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
           <t>discount</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>delivery</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>tax_rate</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>tax_amount</t>
-        </is>
-      </c>
       <c r="P1" t="inlineStr">
         <is>
           <t>total</t>
@@ -528,22 +526,12 @@
       </c>
       <c r="R1" t="inlineStr">
         <is>
-          <t>balance_due</t>
+          <t>deposit date</t>
         </is>
       </c>
       <c r="S1" t="inlineStr">
         <is>
-          <t>line_count</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>lines_match_subtotal</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>total_reconciles</t>
+          <t>balance due</t>
         </is>
       </c>
     </row>
@@ -598,7 +586,7 @@
         <v>20750</v>
       </c>
       <c r="L2" t="n">
-        <v>0</v>
+        <v>3112.5</v>
       </c>
       <c r="M2" t="n">
         <v>0</v>
@@ -607,7 +595,7 @@
         <v>15</v>
       </c>
       <c r="O2" t="n">
-        <v>3112.5</v>
+        <v>0</v>
       </c>
       <c r="P2" t="n">
         <v>23862.5</v>
@@ -615,17 +603,9 @@
       <c r="Q2" t="n">
         <v>0</v>
       </c>
-      <c r="R2" t="n">
+      <c r="R2" t="inlineStr"/>
+      <c r="S2" t="n">
         <v>23862.5</v>
-      </c>
-      <c r="S2" t="n">
-        <v>6</v>
-      </c>
-      <c r="T2" t="b">
-        <v>1</v>
-      </c>
-      <c r="U2" t="b">
-        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -675,7 +655,7 @@
         <v>372267.5</v>
       </c>
       <c r="L3" t="n">
-        <v>0</v>
+        <v>55907.62</v>
       </c>
       <c r="M3" t="n">
         <v>450</v>
@@ -684,7 +664,7 @@
         <v>15</v>
       </c>
       <c r="O3" t="n">
-        <v>55907.62</v>
+        <v>0</v>
       </c>
       <c r="P3" t="n">
         <v>428625.12</v>
@@ -692,17 +672,9 @@
       <c r="Q3" t="n">
         <v>0</v>
       </c>
-      <c r="R3" t="n">
+      <c r="R3" t="inlineStr"/>
+      <c r="S3" t="n">
         <v>428625.12</v>
-      </c>
-      <c r="S3" t="n">
-        <v>32</v>
-      </c>
-      <c r="T3" t="b">
-        <v>1</v>
-      </c>
-      <c r="U3" t="b">
-        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -761,17 +733,9 @@
       <c r="Q4" t="n">
         <v>0</v>
       </c>
-      <c r="R4" t="n">
+      <c r="R4" t="inlineStr"/>
+      <c r="S4" t="n">
         <v>11250</v>
-      </c>
-      <c r="S4" t="n">
-        <v>5</v>
-      </c>
-      <c r="T4" t="b">
-        <v>1</v>
-      </c>
-      <c r="U4" t="b">
-        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -821,7 +785,7 @@
         <v>32000</v>
       </c>
       <c r="L5" t="n">
-        <v>1600</v>
+        <v>4560</v>
       </c>
       <c r="M5" t="n">
         <v>0</v>
@@ -830,7 +794,7 @@
         <v>15</v>
       </c>
       <c r="O5" t="n">
-        <v>4560</v>
+        <v>1600</v>
       </c>
       <c r="P5" t="n">
         <v>34960</v>
@@ -838,17 +802,13 @@
       <c r="Q5" t="n">
         <v>10000</v>
       </c>
-      <c r="R5" t="n">
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="S5" t="n">
         <v>24960</v>
-      </c>
-      <c r="S5" t="n">
-        <v>5</v>
-      </c>
-      <c r="T5" t="b">
-        <v>1</v>
-      </c>
-      <c r="U5" t="b">
-        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -919,17 +879,9 @@
       <c r="Q6" t="n">
         <v>0</v>
       </c>
-      <c r="R6" t="n">
+      <c r="R6" t="inlineStr"/>
+      <c r="S6" t="n">
         <v>313.9</v>
-      </c>
-      <c r="S6" t="n">
-        <v>4</v>
-      </c>
-      <c r="T6" t="b">
-        <v>1</v>
-      </c>
-      <c r="U6" t="b">
-        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -961,12 +913,12 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>source_file</t>
+          <t>source file</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>invoice_number</t>
+          <t>invoice number</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
@@ -976,7 +928,7 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>item_code</t>
+          <t>item code</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
@@ -991,22 +943,22 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>unit_price</t>
+          <t>unit price</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>discount_percent</t>
+          <t>discount percent</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>discount_amount</t>
+          <t>discount amount</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>line_total</t>
+          <t>line total</t>
         </is>
       </c>
     </row>

</xml_diff>